<commit_message>
feat: add CHUNG CƯ RIVA PARK to project list
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="429" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Login" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="CanHo" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="GIAM" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Project" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet name="BaoCao" sheetId="6" state="hidden" r:id="rId6"/>
-    <sheet name="NoCu" sheetId="7" state="hidden" r:id="rId7"/>
-    <sheet name="DaThanhToan" sheetId="8" state="hidden" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CanHo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GIAM" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaoCao" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NoCu" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DaThanhToan" sheetId="8" state="hidden" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Data'!$A$1:$C$223</definedName>
@@ -8423,7 +8423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.88671875" defaultRowHeight="13.8"/>
   <cols>
     <col width="37" customWidth="1" style="11" min="1" max="1"/>
@@ -9811,6 +9811,13 @@
       <c r="I32" t="inlineStr">
         <is>
           <t>04/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>CHUNG CƯ RIVA PARK</t>
         </is>
       </c>
     </row>

</xml_diff>